<commit_message>
add assembly language notes
</commit_message>
<xml_diff>
--- a/Evening/03 Finance For Computer Science/01 Students List/Student_List_Attendance.xlsx
+++ b/Evening/03 Finance For Computer Science/01 Students List/Student_List_Attendance.xlsx
@@ -14,6 +14,9 @@
   <sheets>
     <sheet name="Student List &amp; Attendance" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Student List &amp; Attendance'!$A$4:$D$33</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
@@ -453,16 +456,16 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -775,43 +778,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="9"/>
-      <c r="T1" s="9"/>
-      <c r="U1" s="9"/>
-      <c r="V1" s="9"/>
-      <c r="W1" s="9"/>
-      <c r="X1" s="9"/>
-      <c r="Y1" s="9"/>
-      <c r="Z1" s="9"/>
-      <c r="AA1" s="9"/>
-      <c r="AB1" s="9"/>
-      <c r="AC1" s="9"/>
-      <c r="AD1" s="9"/>
-      <c r="AE1" s="9"/>
-      <c r="AF1" s="9"/>
-      <c r="AG1" s="9"/>
-      <c r="AH1" s="9"/>
-      <c r="AI1" s="9"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="11"/>
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
+      <c r="V1" s="11"/>
+      <c r="W1" s="11"/>
+      <c r="X1" s="11"/>
+      <c r="Y1" s="11"/>
+      <c r="Z1" s="11"/>
+      <c r="AA1" s="11"/>
+      <c r="AB1" s="11"/>
+      <c r="AC1" s="11"/>
+      <c r="AD1" s="11"/>
+      <c r="AE1" s="11"/>
+      <c r="AF1" s="11"/>
+      <c r="AG1" s="11"/>
+      <c r="AH1" s="11"/>
+      <c r="AI1" s="11"/>
     </row>
     <row r="2" spans="1:35" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2141,13 +2144,13 @@
       <c r="AI32" s="6"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="11">
+      <c r="A33" s="9">
         <v>29</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="8" t="s">
         <v>90</v>
       </c>
       <c r="D33" t="s">
@@ -2155,6 +2158,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:D33"/>
   <mergeCells count="1">
     <mergeCell ref="A1:AI1"/>
   </mergeCells>

</xml_diff>